<commit_message>
backup: 20260713_172411 full backup
</commit_message>
<xml_diff>
--- a/建筑行业专家组专家名单.xlsx
+++ b/建筑行业专家组专家名单.xlsx
@@ -104,27 +104,7 @@
     <t>奉贤二建股份公司副总</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">魏 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="楷体_GB2312"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="楷体_GB2312"/>
-        <charset val="134"/>
-      </rPr>
-      <t>东</t>
-    </r>
+    <t>魏  东</t>
   </si>
   <si>
     <t>土木工程</t>
@@ -191,16 +171,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <b/>
-      <sz val="12"/>
+      <sz val="10"/>
       <color theme="1"/>
-      <name val="楷体_GB2312"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="楷体_GB2312"/>
+      <name val="微软雅黑"/>
       <charset val="134"/>
     </font>
     <font>
@@ -813,14 +793,17 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1348,362 +1331,369 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B1:K12"/>
-  <sheetFormatPr defaultColWidth="9.02654867256637" defaultRowHeight="13.5"/>
+  <dimension ref="B2:K12"/>
+  <sheetFormatPr defaultColWidth="9.02654867256637" defaultRowHeight="13.85"/>
   <cols>
-    <col min="11" max="11" width="10.1681415929204"/>
+    <col min="1" max="4" width="9.02654867256637" style="1"/>
+    <col min="5" max="5" width="15.7345132743363" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.8141592920354" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.9557522123894" style="1" customWidth="1"/>
+    <col min="8" max="8" width="9.02654867256637" style="1"/>
+    <col min="9" max="9" width="14.5398230088496" style="1" customWidth="1"/>
+    <col min="10" max="10" width="40.3008849557522" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.5398230088496" style="1"/>
+    <col min="12" max="16384" width="9.02654867256637" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1"/>
-    <row r="2" ht="47.25" spans="2:11">
-      <c r="B2" s="1" t="s">
+    <row r="2" ht="14.65" spans="2:11">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="I2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="K2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" ht="45" spans="2:11">
-      <c r="B3" s="2">
+    <row r="3" ht="13.9" spans="2:11">
+      <c r="B3" s="3">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="I3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="3">
         <v>13501867035</v>
       </c>
     </row>
-    <row r="4" ht="45" spans="2:11">
-      <c r="B4" s="2">
+    <row r="4" ht="13.9" spans="2:11">
+      <c r="B4" s="3">
         <v>2</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="3">
         <v>13321853899</v>
       </c>
     </row>
-    <row r="5" ht="33.75" spans="2:11">
-      <c r="B5" s="2">
+    <row r="5" ht="13.9" spans="2:11">
+      <c r="B5" s="3">
         <v>3</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="3">
         <v>18930196506</v>
       </c>
     </row>
-    <row r="6" ht="22.5" spans="2:11">
-      <c r="B6" s="2">
+    <row r="6" ht="13.9" spans="2:11">
+      <c r="B6" s="3">
         <v>4</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="J6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="3">
         <v>18930196550</v>
       </c>
     </row>
-    <row r="7" ht="33.75" spans="2:11">
-      <c r="B7" s="2">
+    <row r="7" ht="13.9" spans="2:11">
+      <c r="B7" s="3">
         <v>5</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="3">
         <v>18621180090</v>
       </c>
     </row>
-    <row r="8" ht="33.75" spans="2:11">
-      <c r="B8" s="2">
+    <row r="8" ht="13.9" spans="2:11">
+      <c r="B8" s="3">
         <v>6</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="2" t="s">
+      <c r="J8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="3">
         <v>13761874111</v>
       </c>
     </row>
-    <row r="9" ht="33.75" spans="2:11">
-      <c r="B9" s="2">
+    <row r="9" ht="13.9" spans="2:11">
+      <c r="B9" s="3">
         <v>7</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H9" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="I9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J9" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="3">
         <v>13817815049</v>
       </c>
     </row>
-    <row r="10" ht="45" spans="2:11">
-      <c r="B10" s="2">
+    <row r="10" ht="13.9" spans="2:11">
+      <c r="B10" s="3">
         <v>8</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J10" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="3">
         <v>13127931653</v>
       </c>
     </row>
-    <row r="11" ht="45" spans="2:11">
-      <c r="B11" s="2">
+    <row r="11" ht="13.9" spans="2:11">
+      <c r="B11" s="3">
         <v>9</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="H11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="I11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J11" s="2" t="s">
+      <c r="J11" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="3">
         <v>18049828723</v>
       </c>
     </row>
-    <row r="12" ht="22.5" spans="2:11">
-      <c r="B12" s="2">
+    <row r="12" ht="13.9" spans="2:11">
+      <c r="B12" s="3">
         <v>10</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="I12" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J12" s="2" t="s">
+      <c r="J12" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="3">
         <v>13817973866</v>
       </c>
     </row>

</xml_diff>